<commit_message>
Batch 10 SEC tests: SEC-02, SEC-06, SEC-07
</commit_message>
<xml_diff>
--- a/LG_Pilates_Test_Scenarios.xlsx
+++ b/LG_Pilates_Test_Scenarios.xlsx
@@ -2381,17 +2381,17 @@
       </c>
     </row>
     <row r="5" ht="105" customHeight="1" s="82">
-      <c r="A5" s="67" t="inlineStr">
+      <c r="A5" s="92" t="inlineStr">
         <is>
           <t>SEC-03</t>
         </is>
       </c>
-      <c r="B5" s="67" t="inlineStr">
+      <c r="B5" s="92" t="inlineStr">
         <is>
           <t>New-client full booking works end-to-end (anon writes PAR-Q + creates customer/booking via RPCs)</t>
         </is>
       </c>
-      <c r="C5" s="67" t="inlineStr">
+      <c r="C5" s="92" t="inlineStr">
         <is>
           <t>1. In incognito window, book a class as a NEW client
 2. Use email NOT already in the system
@@ -2399,7 +2399,7 @@
 4. Run SQL to verify all three rows were created</t>
         </is>
       </c>
-      <c r="D5" s="67" t="inlineStr">
+      <c r="D5" s="92" t="inlineStr">
         <is>
           <t>- Booking completes successfully
 - customers row created via upsert_customer RPC
@@ -2407,7 +2407,7 @@
 - parq row created via direct anon INSERT (the one retained anon write)</t>
         </is>
       </c>
-      <c r="E5" s="68" t="inlineStr">
+      <c r="E5" s="93" t="inlineStr">
         <is>
           <t>-- Confirm latest customer, booking, and PAR-Q all created:
 SELECT c.id, c.first_name, c.email, c.created_at
@@ -2418,11 +2418,11 @@
 FROM parq ORDER BY id DESC LIMIT 1;</t>
         </is>
       </c>
-      <c r="F5" s="67" t="n"/>
-      <c r="G5" s="67" t="n"/>
-      <c r="H5" s="67" t="inlineStr">
-        <is>
-          <t>Session 5 / audit item 20</t>
+      <c r="F5" s="92" t="n"/>
+      <c r="G5" s="92" t="n"/>
+      <c r="H5" s="92" t="inlineStr">
+        <is>
+          <t>Duplicate of CB-01 — covered by new-client full-flow spec (Session 22, Batch 10)</t>
         </is>
       </c>
     </row>
@@ -2529,9 +2529,10 @@
       <c r="C8" s="69" t="inlineStr">
         <is>
           <t>1. Sign in to admin dashboard with Louise's credentials
-2. Verify every tab loads: All Bookings, By Class, Clients,
-   Cancellations, Settings, Backup &amp; Export
-3. Try each primary admin action:
+2. Verify all 4 dashboard tabs load: All Bookings, By Class, Clients, Cancellations
+3. Verify the 3 below-tab sections render: Upcoming Classes,
+   Settings, Backup &amp; Export
+4. Try each primary admin action:
    - Confirm a booking
    - Add/edit/delete a class
    - View a PAR-Q
@@ -2540,7 +2541,8 @@
       </c>
       <c r="D8" s="69" t="inlineStr">
         <is>
-          <t>- All tabs load without errors
+          <t>- All 4 tabs load without errors
+- All 3 below-tab sections render their headings and primary controls
 - All CRUD actions succeed
 - Confirms authenticated role retains full privileges
   (item 20 changes did not affect admin)</t>

</xml_diff>

<commit_message>
Batch 11 complete — Edge Cases part 1 (6 EC specs)
</commit_message>
<xml_diff>
--- a/LG_Pilates_Test_Scenarios.xlsx
+++ b/LG_Pilates_Test_Scenarios.xlsx
@@ -1430,7 +1430,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1. Run the SQL to archive all blocks temporarily
+          <t>1. Run the SQL to hide all active and upcoming blocks from public view
 2. Reload the public booking page
 3. Restore blocks after</t>
         </is>
@@ -1443,18 +1443,19 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>-- Archive all blocks:
-UPDATE blocks SET status = 'archived';
+          <t>-- Hide all active and upcoming blocks from public view:
+UPDATE blocks SET visible = false
+WHERE status IN ('active','upcoming');
 -- Restore after test:
-UPDATE blocks SET status = 'upcoming'
-WHERE start_date &gt;= CURRENT_DATE;</t>
+UPDATE blocks SET visible = true
+WHERE status IN ('active','upcoming');</t>
         </is>
       </c>
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Restore immediately after</t>
+          <t>Use the `visible` column to hide blocks from the public grid — front-end filter in getActiveBlock() is `visible !== false`, NOT status. Restore immediately after.</t>
         </is>
       </c>
     </row>
@@ -1471,20 +1472,27 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1. Enter 100+ characters in the name field
-2. Complete the booking</t>
+          <t>1. Open the booking modal
+2. Try to enter 100+ characters in the First Name field
+3. Complete the booking</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
           <t>- Handled gracefully — no crash
-- No layout breakage in admin dashboard rows</t>
+- First Name input caps at 50 characters (maxlength=50)
+- Booking completes successfully with the truncated name
+- No layout breakage in the admin Bookings table row</t>
         </is>
       </c>
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>The b-firstname input has maxlength="50" so the browser physically prevents typing past 50 chars. The test verifies the cap is enforced and the booking flow handles the truncated name end-to-end.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="84" customHeight="1" s="82">
       <c r="A9" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Batch 15 AB tests: AB-02, AB-03, AB-04, AB-05/06, AB-07
</commit_message>
<xml_diff>
--- a/LG_Pilates_Test_Scenarios.xlsx
+++ b/LG_Pilates_Test_Scenarios.xlsx
@@ -4906,33 +4906,33 @@
       </c>
     </row>
     <row r="3" ht="105" customHeight="1" s="82">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="89" t="inlineStr">
         <is>
           <t>AB-01</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="90" t="inlineStr">
         <is>
           <t>Admin can log in</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="90" t="inlineStr">
         <is>
           <t>1. Click Dashboard in nav bar
 2. Enter email and password
 3. Click Sign In</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="90" t="inlineStr">
         <is>
           <t>- Dashboard loads with stats and tabs
 - No error message shown</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+      <c r="E3" s="90" t="n"/>
+      <c r="F3" s="90" t="n"/>
+      <c r="G3" s="90" t="n"/>
+      <c r="H3" s="90" t="n"/>
     </row>
     <row r="4" ht="105" customHeight="1" s="82">
       <c r="A4" s="5" t="inlineStr">

</xml_diff>